<commit_message>
Third instance of the merge-key collapse: 31 rows lost
WCO Loss Runs 2018-2022.PDF joins the list — 8 raw rows, one distinct key
('0196-47556', '', ''), one row shipped. Two of the three affected
documents collapse to a single row.

Also notes the distinction the metric was blurring: Reaco - 2022 WC - LR
collapses 24 raw rows to 12 and that is correct deduplication, not loss.
Which it is, is exactly what MergeResult.conflicts records and
finalize_rows throws away.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparisons/_all.xlsx
+++ b/comparisons/_all.xlsx
@@ -666,73 +666,73 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="E3" t="n">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="F3" t="n">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="G3" t="n">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="H3" t="n">
-        <v>87.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="I3" t="n">
         <v>92.5</v>
       </c>
       <c r="J3" t="n">
-        <v>86.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>75.5</v>
+        <v>75.3</v>
       </c>
       <c r="L3" t="n">
-        <v>7107</v>
+        <v>7292</v>
       </c>
       <c r="M3" t="n">
-        <v>6154</v>
+        <v>6295</v>
       </c>
       <c r="N3" t="n">
-        <v>86.59</v>
+        <v>86.33</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="P3" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="Q3" t="n">
-        <v>1080132</v>
+        <v>1156252</v>
       </c>
       <c r="R3" t="n">
-        <v>546254</v>
+        <v>625762</v>
       </c>
       <c r="S3" t="n">
-        <v>0.216</v>
+        <v>0.2313</v>
       </c>
       <c r="T3" t="n">
-        <v>0.437</v>
+        <v>0.5006</v>
       </c>
       <c r="U3" t="n">
-        <v>0.653</v>
+        <v>0.7319</v>
       </c>
       <c r="V3" t="n">
-        <v>0.005062</v>
+        <v>0.005381</v>
       </c>
       <c r="W3" t="n">
-        <v>0.001741</v>
+        <v>0.001901</v>
       </c>
       <c r="X3" t="n">
-        <v>2197.4</v>
+        <v>2206.7</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AA28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1821,16 +1821,16 @@
         <v>6.2</v>
       </c>
       <c r="K12" t="n">
-        <v>63.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="M12" t="n">
-        <v>63.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="N12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O12" t="n">
         <v>19</v>
@@ -2402,20 +2402,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Loss Runs Report 5 years recent.pdf</t>
+          <t>DetailResults_ACP_3086469186.pdf</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -2430,55 +2430,55 @@
         <v>100</v>
       </c>
       <c r="K19" t="n">
-        <v>76.2</v>
+        <v>60</v>
       </c>
       <c r="L19" t="n">
-        <v>76.2</v>
+        <v>60</v>
       </c>
       <c r="M19" t="n">
-        <v>76.2</v>
+        <v>60</v>
       </c>
       <c r="N19" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="O19" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R19" t="n">
-        <v>64691</v>
+        <v>27169</v>
       </c>
       <c r="S19" t="n">
-        <v>5342</v>
+        <v>12728</v>
       </c>
       <c r="T19" t="n">
-        <v>10782</v>
+        <v>9056</v>
       </c>
       <c r="U19" t="n">
-        <v>890</v>
+        <v>4243</v>
       </c>
       <c r="V19" t="n">
-        <v>0.012938</v>
+        <v>0.005434</v>
       </c>
       <c r="W19" t="n">
-        <v>0.004274</v>
+        <v>0.010183</v>
       </c>
       <c r="X19" t="n">
-        <v>0.017212</v>
+        <v>0.015616</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.002869</v>
+        <v>0.005205</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.008606000000000001</v>
+        <v>0.015616</v>
       </c>
       <c r="AA19" t="n">
-        <v>56.2</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20">
@@ -2489,17 +2489,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>GLI Loss Runs.PDF</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
         <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>5</v>
@@ -2514,58 +2514,58 @@
         <v>100</v>
       </c>
       <c r="J20" t="n">
-        <v>71.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="K20" t="n">
-        <v>94.5</v>
+        <v>65.7</v>
       </c>
       <c r="L20" t="n">
-        <v>94.5</v>
+        <v>65.7</v>
       </c>
       <c r="M20" t="n">
-        <v>94.5</v>
+        <v>65.7</v>
       </c>
       <c r="N20" t="n">
-        <v>104</v>
+        <v>65</v>
       </c>
       <c r="O20" t="n">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R20" t="n">
-        <v>34345</v>
+        <v>22697</v>
       </c>
       <c r="S20" t="n">
-        <v>18350</v>
+        <v>44907</v>
       </c>
       <c r="T20" t="n">
-        <v>8586</v>
+        <v>11348</v>
       </c>
       <c r="U20" t="n">
-        <v>4588</v>
+        <v>22454</v>
       </c>
       <c r="V20" t="n">
-        <v>0.006869</v>
+        <v>0.004539</v>
       </c>
       <c r="W20" t="n">
-        <v>0.01468</v>
+        <v>0.035926</v>
       </c>
       <c r="X20" t="n">
-        <v>0.021549</v>
+        <v>0.040465</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.005387</v>
+        <v>0.020233</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.003078</v>
+        <v>0.008092999999999999</v>
       </c>
       <c r="AA20" t="n">
-        <v>49523.2</v>
+        <v>313.8</v>
       </c>
     </row>
     <row r="21">
@@ -2576,83 +2576,83 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>LossRunsReport_9_7_2022.pdf</t>
+          <t>GLI PKG CPP WCO Loss Runs 2017-2018.PDF</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>127</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
-        <v>127</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>127</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="J21" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="K21" t="n">
-        <v>90.8</v>
+        <v>95.5</v>
       </c>
       <c r="L21" t="n">
-        <v>90.8</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>90.8</v>
+        <v>95.5</v>
       </c>
       <c r="N21" t="n">
-        <v>2535</v>
+        <v>63</v>
       </c>
       <c r="O21" t="n">
-        <v>2791</v>
+        <v>66</v>
       </c>
       <c r="P21" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Q21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R21" t="n">
-        <v>284926</v>
+        <v>26254</v>
       </c>
       <c r="S21" t="n">
-        <v>51691</v>
+        <v>21873</v>
       </c>
       <c r="T21" t="n">
-        <v>7915</v>
+        <v>13127</v>
       </c>
       <c r="U21" t="n">
-        <v>1436</v>
+        <v>10936</v>
       </c>
       <c r="V21" t="n">
-        <v>0.056986</v>
+        <v>0.005251</v>
       </c>
       <c r="W21" t="n">
-        <v>0.041353</v>
+        <v>0.017498</v>
       </c>
       <c r="X21" t="n">
-        <v>0.09833799999999999</v>
+        <v>0.022749</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.002732</v>
+        <v>0.011374</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.0007739999999999999</v>
+        <v>0.005687</v>
       </c>
       <c r="AA21" t="n">
-        <v>311.8</v>
+        <v>149.7</v>
       </c>
     </row>
     <row r="22">
@@ -2663,20 +2663,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Reaco - 2022 Auto - LR_17-20.pdf</t>
+          <t>Loss Runs Report 5 years recent.pdf</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -2688,58 +2688,58 @@
         <v>100</v>
       </c>
       <c r="J22" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="K22" t="n">
-        <v>83.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="L22" t="n">
-        <v>83.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="M22" t="n">
-        <v>83.59999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="N22" t="n">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="O22" t="n">
-        <v>110</v>
+        <v>42</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R22" t="n">
-        <v>38129</v>
+        <v>64691</v>
       </c>
       <c r="S22" t="n">
-        <v>22908</v>
+        <v>5342</v>
       </c>
       <c r="T22" t="n">
-        <v>7626</v>
+        <v>10782</v>
       </c>
       <c r="U22" t="n">
-        <v>4582</v>
+        <v>890</v>
       </c>
       <c r="V22" t="n">
-        <v>0.007626</v>
+        <v>0.012938</v>
       </c>
       <c r="W22" t="n">
-        <v>0.018327</v>
+        <v>0.004274</v>
       </c>
       <c r="X22" t="n">
-        <v>0.025953</v>
+        <v>0.017212</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.005191</v>
+        <v>0.002869</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.004326</v>
+        <v>0.008606000000000001</v>
       </c>
       <c r="AA22" t="n">
-        <v>170.3</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="23">
@@ -2750,20 +2750,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Reaco - 2022 Auto - LR_20-22.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -2775,58 +2775,58 @@
         <v>100</v>
       </c>
       <c r="J23" t="n">
-        <v>100</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K23" t="n">
-        <v>80</v>
+        <v>94.5</v>
       </c>
       <c r="L23" t="n">
-        <v>80</v>
+        <v>94.5</v>
       </c>
       <c r="M23" t="n">
-        <v>80</v>
+        <v>94.5</v>
       </c>
       <c r="N23" t="n">
-        <v>16</v>
+        <v>104</v>
       </c>
       <c r="O23" t="n">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="R23" t="n">
-        <v>12015</v>
+        <v>34345</v>
       </c>
       <c r="S23" t="n">
-        <v>5928</v>
+        <v>18350</v>
       </c>
       <c r="T23" t="n">
-        <v>12015</v>
+        <v>8586</v>
       </c>
       <c r="U23" t="n">
-        <v>5928</v>
+        <v>4588</v>
       </c>
       <c r="V23" t="n">
-        <v>0.002403</v>
+        <v>0.006869</v>
       </c>
       <c r="W23" t="n">
-        <v>0.004743</v>
+        <v>0.01468</v>
       </c>
       <c r="X23" t="n">
-        <v>0.007146</v>
+        <v>0.021549</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.007146</v>
+        <v>0.005387</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.007146</v>
+        <v>0.003078</v>
       </c>
       <c r="AA23" t="n">
-        <v>49.3</v>
+        <v>49523.2</v>
       </c>
     </row>
     <row r="24">
@@ -2837,20 +2837,20 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>LossRunsReport_9_7_2022.pdf</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="D24" t="n">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="E24" t="n">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="F24" t="n">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -2865,55 +2865,55 @@
         <v>100</v>
       </c>
       <c r="K24" t="n">
-        <v>94.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="L24" t="n">
-        <v>94.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="M24" t="n">
-        <v>95</v>
+        <v>90.8</v>
       </c>
       <c r="N24" t="n">
-        <v>245</v>
+        <v>2535</v>
       </c>
       <c r="O24" t="n">
-        <v>258</v>
+        <v>2791</v>
       </c>
       <c r="P24" t="n">
-        <v>8.300000000000001</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R24" t="n">
-        <v>89576</v>
+        <v>284926</v>
       </c>
       <c r="S24" t="n">
-        <v>33117</v>
+        <v>51691</v>
       </c>
       <c r="T24" t="n">
-        <v>3895</v>
+        <v>7915</v>
       </c>
       <c r="U24" t="n">
-        <v>1440</v>
+        <v>1436</v>
       </c>
       <c r="V24" t="n">
-        <v>0.017915</v>
+        <v>0.056986</v>
       </c>
       <c r="W24" t="n">
-        <v>0.026493</v>
+        <v>0.041353</v>
       </c>
       <c r="X24" t="n">
-        <v>0.044409</v>
+        <v>0.09833799999999999</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.001931</v>
+        <v>0.002732</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.003701</v>
+        <v>0.0007739999999999999</v>
       </c>
       <c r="AA24" t="n">
-        <v>31956.9</v>
+        <v>311.8</v>
       </c>
     </row>
     <row r="25">
@@ -2924,17 +2924,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>WC Loss Runs.pdf</t>
+          <t>Reaco - 2022 Auto - LR_17-20.pdf</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D25" t="n">
         <v>5</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
         <v>5</v>
@@ -2949,22 +2949,22 @@
         <v>100</v>
       </c>
       <c r="J25" t="n">
-        <v>100</v>
+        <v>83.3</v>
       </c>
       <c r="K25" t="n">
-        <v>82.40000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="L25" t="n">
-        <v>82.40000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="M25" t="n">
-        <v>82.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="N25" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="O25" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -2973,33 +2973,294 @@
         <v>2</v>
       </c>
       <c r="R25" t="n">
+        <v>38129</v>
+      </c>
+      <c r="S25" t="n">
+        <v>22908</v>
+      </c>
+      <c r="T25" t="n">
+        <v>7626</v>
+      </c>
+      <c r="U25" t="n">
+        <v>4582</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0.007626</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.018327</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.025953</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0.005191</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0.004326</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>170.3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Reaco - 2022 Auto - LR_20-22.pdf</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="n">
+        <v>100</v>
+      </c>
+      <c r="K26" t="n">
+        <v>80</v>
+      </c>
+      <c r="L26" t="n">
+        <v>80</v>
+      </c>
+      <c r="M26" t="n">
+        <v>80</v>
+      </c>
+      <c r="N26" t="n">
+        <v>16</v>
+      </c>
+      <c r="O26" t="n">
+        <v>20</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>2</v>
+      </c>
+      <c r="R26" t="n">
+        <v>12015</v>
+      </c>
+      <c r="S26" t="n">
+        <v>5928</v>
+      </c>
+      <c r="T26" t="n">
+        <v>12015</v>
+      </c>
+      <c r="U26" t="n">
+        <v>5928</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.002403</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.004743</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0.007146</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0.007146</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0.007146</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>49.3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Reaco - 2022 WC - LR.pdf</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>23</v>
+      </c>
+      <c r="D27" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" t="n">
+        <v>12</v>
+      </c>
+      <c r="F27" t="n">
+        <v>12</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="n">
+        <v>100</v>
+      </c>
+      <c r="K27" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="L27" t="n">
+        <v>94.90000000000001</v>
+      </c>
+      <c r="M27" t="n">
+        <v>95</v>
+      </c>
+      <c r="N27" t="n">
+        <v>245</v>
+      </c>
+      <c r="O27" t="n">
+        <v>258</v>
+      </c>
+      <c r="P27" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>7</v>
+      </c>
+      <c r="R27" t="n">
+        <v>89576</v>
+      </c>
+      <c r="S27" t="n">
+        <v>33117</v>
+      </c>
+      <c r="T27" t="n">
+        <v>3895</v>
+      </c>
+      <c r="U27" t="n">
+        <v>1440</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.017915</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.026493</v>
+      </c>
+      <c r="X27" t="n">
+        <v>0.044409</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0.001931</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0.003701</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>31956.9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>WC Loss Runs.pdf</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="n">
+        <v>100</v>
+      </c>
+      <c r="K28" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="L28" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="M28" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="N28" t="n">
+        <v>94</v>
+      </c>
+      <c r="O28" t="n">
+        <v>114</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>2</v>
+      </c>
+      <c r="R28" t="n">
         <v>39337</v>
       </c>
-      <c r="S25" t="n">
+      <c r="S28" t="n">
         <v>21431</v>
       </c>
-      <c r="T25" t="n">
+      <c r="T28" t="n">
         <v>6556</v>
       </c>
-      <c r="U25" t="n">
+      <c r="U28" t="n">
         <v>3572</v>
       </c>
-      <c r="V25" t="n">
+      <c r="V28" t="n">
         <v>0.007868</v>
       </c>
-      <c r="W25" t="n">
+      <c r="W28" t="n">
         <v>0.017145</v>
       </c>
-      <c r="X25" t="n">
+      <c r="X28" t="n">
         <v>0.025013</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="Y28" t="n">
         <v>0.004169</v>
       </c>
-      <c r="Z25" t="n">
+      <c r="Z28" t="n">
         <v>0.005003</v>
       </c>
-      <c r="AA25" t="n">
+      <c r="AA28" t="n">
         <v>153.1</v>
       </c>
     </row>
@@ -3014,7 +3275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P86"/>
+  <dimension ref="A1:P92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6901,7 +7162,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Loss Runs Report 5 years recent.pdf</t>
+          <t>DetailResults_ACP_3086469186.pdf</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -6921,11 +7182,11 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -6933,28 +7194,28 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>20.02</v>
+        <v>14.8</v>
       </c>
       <c r="J61" t="n">
-        <v>19182</v>
+        <v>13413</v>
       </c>
       <c r="K61" t="n">
-        <v>1472</v>
+        <v>1361</v>
       </c>
       <c r="L61" t="n">
-        <v>3836</v>
+        <v>4471</v>
       </c>
       <c r="M61" t="n">
-        <v>294</v>
+        <v>454</v>
       </c>
       <c r="N61" t="n">
-        <v>0.003836</v>
+        <v>0.002683</v>
       </c>
       <c r="O61" t="n">
-        <v>0.001178</v>
+        <v>0.001089</v>
       </c>
       <c r="P61" t="n">
-        <v>0.005014</v>
+        <v>0.003771</v>
       </c>
     </row>
     <row r="62">
@@ -6965,7 +7226,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Loss Runs Report 5 years recent.pdf</t>
+          <t>DetailResults_ACP_3086469186.pdf</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -6985,11 +7246,11 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>1-6</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -6997,28 +7258,28 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>16.1</v>
+        <v>81.02</v>
       </c>
       <c r="J62" t="n">
-        <v>22629</v>
+        <v>13756</v>
       </c>
       <c r="K62" t="n">
-        <v>1785</v>
+        <v>11367</v>
       </c>
       <c r="L62" t="n">
-        <v>3772</v>
+        <v>4585</v>
       </c>
       <c r="M62" t="n">
-        <v>298</v>
+        <v>3789</v>
       </c>
       <c r="N62" t="n">
-        <v>0.004526</v>
+        <v>0.002751</v>
       </c>
       <c r="O62" t="n">
-        <v>0.001428</v>
+        <v>0.009094</v>
       </c>
       <c r="P62" t="n">
-        <v>0.005954</v>
+        <v>0.011845</v>
       </c>
     </row>
     <row r="63">
@@ -7029,12 +7290,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Loss Runs Report 5 years recent.pdf</t>
+          <t>GLI Loss Runs.PDF</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7044,16 +7305,16 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>1-6</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
@@ -7061,28 +7322,28 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>19.9</v>
+        <v>15.44</v>
       </c>
       <c r="J63" t="n">
-        <v>22880</v>
+        <v>11126</v>
       </c>
       <c r="K63" t="n">
-        <v>2085</v>
+        <v>1460</v>
       </c>
       <c r="L63" t="n">
-        <v>3813</v>
+        <v>5563</v>
       </c>
       <c r="M63" t="n">
-        <v>348</v>
+        <v>730</v>
       </c>
       <c r="N63" t="n">
-        <v>0.004576</v>
+        <v>0.002225</v>
       </c>
       <c r="O63" t="n">
-        <v>0.001668</v>
+        <v>0.001168</v>
       </c>
       <c r="P63" t="n">
-        <v>0.006244</v>
+        <v>0.003393</v>
       </c>
     </row>
     <row r="64">
@@ -7093,12 +7354,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>GLI Loss Runs.PDF</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7108,16 +7369,16 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -7125,28 +7386,28 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>16.58</v>
+        <v>298.16</v>
       </c>
       <c r="J64" t="n">
-        <v>16959</v>
+        <v>11571</v>
       </c>
       <c r="K64" t="n">
-        <v>1355</v>
+        <v>43447</v>
       </c>
       <c r="L64" t="n">
-        <v>4240</v>
+        <v>5786</v>
       </c>
       <c r="M64" t="n">
-        <v>339</v>
+        <v>21724</v>
       </c>
       <c r="N64" t="n">
-        <v>0.003392</v>
+        <v>0.002314</v>
       </c>
       <c r="O64" t="n">
-        <v>0.001084</v>
+        <v>0.034758</v>
       </c>
       <c r="P64" t="n">
-        <v>0.004476</v>
+        <v>0.037072</v>
       </c>
     </row>
     <row r="65">
@@ -7157,12 +7418,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>GLI PKG CPP WCO Loss Runs 2017-2018.PDF</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7172,16 +7433,16 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
@@ -7189,28 +7450,28 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>118.37</v>
+        <v>18.88</v>
       </c>
       <c r="J65" t="n">
-        <v>17386</v>
+        <v>12906</v>
       </c>
       <c r="K65" t="n">
-        <v>16995</v>
+        <v>1915</v>
       </c>
       <c r="L65" t="n">
-        <v>4346</v>
+        <v>6453</v>
       </c>
       <c r="M65" t="n">
-        <v>4249</v>
+        <v>958</v>
       </c>
       <c r="N65" t="n">
-        <v>0.003477</v>
+        <v>0.002581</v>
       </c>
       <c r="O65" t="n">
-        <v>0.013596</v>
+        <v>0.001532</v>
       </c>
       <c r="P65" t="n">
-        <v>0.017073</v>
+        <v>0.004113</v>
       </c>
     </row>
     <row r="66">
@@ -7221,12 +7482,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>GLI PKG CPP WCO Loss Runs 2017-2018.PDF</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7241,40 +7502,40 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>294.39</v>
+        <v>130.58</v>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>13348</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>19958</v>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
+        <v>6674</v>
       </c>
       <c r="M66" t="n">
-        <v>0</v>
+        <v>9979</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>0.00267</v>
       </c>
       <c r="O66" t="n">
-        <v>0</v>
+        <v>0.015966</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>0.018636</v>
       </c>
     </row>
     <row r="67">
@@ -7285,12 +7546,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>Loss Runs Report 5 years recent.pdf</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7300,45 +7561,45 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="G67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>136.46</v>
+        <v>20.02</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>19182</v>
       </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>1472</v>
       </c>
       <c r="L67" t="n">
-        <v>0</v>
+        <v>3836</v>
       </c>
       <c r="M67" t="n">
-        <v>0</v>
+        <v>294</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>0.003836</v>
       </c>
       <c r="O67" t="n">
-        <v>0</v>
+        <v>0.001178</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>0.005014</v>
       </c>
     </row>
     <row r="68">
@@ -7349,12 +7610,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>Loss Runs Report 5 years recent.pdf</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7369,40 +7630,40 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-6</t>
         </is>
       </c>
       <c r="G68" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>38.81</v>
+        <v>16.1</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>22629</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>1785</v>
       </c>
       <c r="L68" t="n">
-        <v>0</v>
+        <v>3772</v>
       </c>
       <c r="M68" t="n">
-        <v>0</v>
+        <v>298</v>
       </c>
       <c r="N68" t="n">
-        <v>0</v>
+        <v>0.004526</v>
       </c>
       <c r="O68" t="n">
-        <v>0</v>
+        <v>0.001428</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>0.005954</v>
       </c>
     </row>
     <row r="69">
@@ -7413,7 +7674,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Loss Runs.pdf</t>
+          <t>Loss Runs Report 5 years recent.pdf</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -7433,40 +7694,40 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-6</t>
         </is>
       </c>
       <c r="G69" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>0.16</v>
+        <v>19.9</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>22880</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>2085</v>
       </c>
       <c r="L69" t="n">
-        <v>0</v>
+        <v>3813</v>
       </c>
       <c r="M69" t="n">
-        <v>0</v>
+        <v>348</v>
       </c>
       <c r="N69" t="n">
-        <v>0</v>
+        <v>0.004576</v>
       </c>
       <c r="O69" t="n">
-        <v>0</v>
+        <v>0.001668</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>0.006244</v>
       </c>
     </row>
     <row r="70">
@@ -7482,7 +7743,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7492,7 +7753,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -7505,32 +7766,32 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>149.5</v>
+        <v>16.58</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>16959</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>1355</v>
       </c>
       <c r="L70" t="n">
-        <v>0</v>
+        <v>4240</v>
       </c>
       <c r="M70" t="n">
-        <v>0</v>
+        <v>339</v>
       </c>
       <c r="N70" t="n">
-        <v>0</v>
+        <v>0.003392</v>
       </c>
       <c r="O70" t="n">
-        <v>0</v>
+        <v>0.001084</v>
       </c>
       <c r="P70" t="n">
-        <v>0</v>
+        <v>0.004476</v>
       </c>
     </row>
     <row r="71">
@@ -7541,12 +7802,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>LossRunsReport_9_7_2022.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7556,16 +7817,16 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
@@ -7573,28 +7834,28 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>16.34</v>
+        <v>118.37</v>
       </c>
       <c r="J71" t="n">
-        <v>21243</v>
+        <v>17386</v>
       </c>
       <c r="K71" t="n">
-        <v>1382</v>
+        <v>16995</v>
       </c>
       <c r="L71" t="n">
+        <v>4346</v>
+      </c>
+      <c r="M71" t="n">
         <v>4249</v>
       </c>
-      <c r="M71" t="n">
-        <v>276</v>
-      </c>
       <c r="N71" t="n">
-        <v>0.004249</v>
+        <v>0.003477</v>
       </c>
       <c r="O71" t="n">
-        <v>0.001106</v>
+        <v>0.013596</v>
       </c>
       <c r="P71" t="n">
-        <v>0.005354</v>
+        <v>0.017073</v>
       </c>
     </row>
     <row r="72">
@@ -7605,12 +7866,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>LossRunsReport_9_7_2022.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7625,40 +7886,40 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>1-36</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G72" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>error</t>
         </is>
       </c>
       <c r="I72" t="n">
-        <v>139.2</v>
+        <v>294.39</v>
       </c>
       <c r="J72" t="n">
-        <v>123635</v>
+        <v>0</v>
       </c>
       <c r="K72" t="n">
-        <v>28694</v>
+        <v>0</v>
       </c>
       <c r="L72" t="n">
-        <v>3434</v>
+        <v>0</v>
       </c>
       <c r="M72" t="n">
-        <v>797</v>
+        <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>0.024727</v>
+        <v>0</v>
       </c>
       <c r="O72" t="n">
-        <v>0.022955</v>
+        <v>0</v>
       </c>
       <c r="P72" t="n">
-        <v>0.047682</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -7669,7 +7930,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>LossRunsReport_9_7_2022.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -7689,40 +7950,40 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>1-36</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G73" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>error</t>
         </is>
       </c>
       <c r="I73" t="n">
-        <v>155.94</v>
+        <v>136.46</v>
       </c>
       <c r="J73" t="n">
-        <v>140048</v>
+        <v>0</v>
       </c>
       <c r="K73" t="n">
-        <v>21615</v>
+        <v>0</v>
       </c>
       <c r="L73" t="n">
-        <v>3890</v>
+        <v>0</v>
       </c>
       <c r="M73" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>0.02801</v>
+        <v>0</v>
       </c>
       <c r="O73" t="n">
-        <v>0.017292</v>
+        <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>0.045302</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -7733,12 +7994,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Reaco - 2022 Auto - LR_17-20.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7748,45 +8009,45 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>error</t>
         </is>
       </c>
       <c r="I74" t="n">
-        <v>17.98</v>
+        <v>38.81</v>
       </c>
       <c r="J74" t="n">
-        <v>18845</v>
+        <v>0</v>
       </c>
       <c r="K74" t="n">
-        <v>1912</v>
+        <v>0</v>
       </c>
       <c r="L74" t="n">
-        <v>3769</v>
+        <v>0</v>
       </c>
       <c r="M74" t="n">
-        <v>382</v>
+        <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>0.003769</v>
+        <v>0</v>
       </c>
       <c r="O74" t="n">
-        <v>0.00153</v>
+        <v>0</v>
       </c>
       <c r="P74" t="n">
-        <v>0.005299</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -7797,12 +8058,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Reaco - 2022 Auto - LR_17-20.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7817,40 +8078,40 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>error</t>
         </is>
       </c>
       <c r="I75" t="n">
-        <v>152.1</v>
+        <v>0.16</v>
       </c>
       <c r="J75" t="n">
-        <v>19284</v>
+        <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>20996</v>
+        <v>0</v>
       </c>
       <c r="L75" t="n">
-        <v>3857</v>
+        <v>0</v>
       </c>
       <c r="M75" t="n">
-        <v>4199</v>
+        <v>0</v>
       </c>
       <c r="N75" t="n">
-        <v>0.003857</v>
+        <v>0</v>
       </c>
       <c r="O75" t="n">
-        <v>0.016797</v>
+        <v>0</v>
       </c>
       <c r="P75" t="n">
-        <v>0.020654</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -7861,12 +8122,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Reaco - 2022 Auto - LR_20-22.pdf</t>
+          <t>Loss Runs.pdf</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7876,45 +8137,45 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>error</t>
         </is>
       </c>
       <c r="I76" t="n">
-        <v>14.59</v>
+        <v>149.5</v>
       </c>
       <c r="J76" t="n">
-        <v>5851</v>
+        <v>0</v>
       </c>
       <c r="K76" t="n">
-        <v>1327</v>
+        <v>0</v>
       </c>
       <c r="L76" t="n">
-        <v>5851</v>
+        <v>0</v>
       </c>
       <c r="M76" t="n">
-        <v>1327</v>
+        <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>0.00117</v>
+        <v>0</v>
       </c>
       <c r="O76" t="n">
-        <v>0.001062</v>
+        <v>0</v>
       </c>
       <c r="P76" t="n">
-        <v>0.002232</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -7925,12 +8186,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Reaco - 2022 Auto - LR_20-22.pdf</t>
+          <t>LossRunsReport_9_7_2022.pdf</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7940,16 +8201,16 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="G77" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
@@ -7957,28 +8218,28 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>34.51</v>
+        <v>16.34</v>
       </c>
       <c r="J77" t="n">
-        <v>6164</v>
+        <v>21243</v>
       </c>
       <c r="K77" t="n">
-        <v>4601</v>
+        <v>1382</v>
       </c>
       <c r="L77" t="n">
-        <v>6164</v>
+        <v>4249</v>
       </c>
       <c r="M77" t="n">
-        <v>4601</v>
+        <v>276</v>
       </c>
       <c r="N77" t="n">
-        <v>0.001233</v>
+        <v>0.004249</v>
       </c>
       <c r="O77" t="n">
-        <v>0.003681</v>
+        <v>0.001106</v>
       </c>
       <c r="P77" t="n">
-        <v>0.004914</v>
+        <v>0.005354</v>
       </c>
     </row>
     <row r="78">
@@ -7989,12 +8250,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>LossRunsReport_9_7_2022.pdf</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8004,16 +8265,16 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-36</t>
         </is>
       </c>
       <c r="G78" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
@@ -8021,28 +8282,28 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>23.95</v>
+        <v>139.2</v>
       </c>
       <c r="J78" t="n">
-        <v>19042</v>
+        <v>123635</v>
       </c>
       <c r="K78" t="n">
-        <v>1933</v>
+        <v>28694</v>
       </c>
       <c r="L78" t="n">
-        <v>3808</v>
+        <v>3434</v>
       </c>
       <c r="M78" t="n">
-        <v>387</v>
+        <v>797</v>
       </c>
       <c r="N78" t="n">
-        <v>0.003808</v>
+        <v>0.024727</v>
       </c>
       <c r="O78" t="n">
-        <v>0.001546</v>
+        <v>0.022955</v>
       </c>
       <c r="P78" t="n">
-        <v>0.005355</v>
+        <v>0.047682</v>
       </c>
     </row>
     <row r="79">
@@ -8053,12 +8314,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>LossRunsReport_9_7_2022.pdf</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>extract</t>
+          <t>qa</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8073,11 +8334,11 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>1-23</t>
+          <t>1-36</t>
         </is>
       </c>
       <c r="G79" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
@@ -8085,28 +8346,28 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>203.15</v>
+        <v>155.94</v>
       </c>
       <c r="J79" t="n">
-        <v>70534</v>
+        <v>140048</v>
       </c>
       <c r="K79" t="n">
-        <v>31184</v>
+        <v>21615</v>
       </c>
       <c r="L79" t="n">
-        <v>3067</v>
+        <v>3890</v>
       </c>
       <c r="M79" t="n">
-        <v>1356</v>
+        <v>600</v>
       </c>
       <c r="N79" t="n">
-        <v>0.014107</v>
+        <v>0.02801</v>
       </c>
       <c r="O79" t="n">
-        <v>0.024947</v>
+        <v>0.017292</v>
       </c>
       <c r="P79" t="n">
-        <v>0.039054</v>
+        <v>0.045302</v>
       </c>
     </row>
     <row r="80">
@@ -8117,12 +8378,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>Reaco - 2022 Auto - LR_17-20.pdf</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8132,45 +8393,45 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>1-23</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="G80" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I80" t="n">
-        <v>104.97</v>
+        <v>17.98</v>
       </c>
       <c r="J80" t="n">
-        <v>0</v>
+        <v>18845</v>
       </c>
       <c r="K80" t="n">
-        <v>0</v>
+        <v>1912</v>
       </c>
       <c r="L80" t="n">
-        <v>0</v>
+        <v>3769</v>
       </c>
       <c r="M80" t="n">
-        <v>0</v>
+        <v>382</v>
       </c>
       <c r="N80" t="n">
-        <v>0</v>
+        <v>0.003769</v>
       </c>
       <c r="O80" t="n">
-        <v>0</v>
+        <v>0.00153</v>
       </c>
       <c r="P80" t="n">
-        <v>0</v>
+        <v>0.005299</v>
       </c>
     </row>
     <row r="81">
@@ -8181,12 +8442,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>Reaco - 2022 Auto - LR_17-20.pdf</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8201,40 +8462,40 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>1-23</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="G81" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I81" t="n">
-        <v>136.66</v>
+        <v>152.1</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>19284</v>
       </c>
       <c r="K81" t="n">
-        <v>0</v>
+        <v>20996</v>
       </c>
       <c r="L81" t="n">
-        <v>0</v>
+        <v>3857</v>
       </c>
       <c r="M81" t="n">
-        <v>0</v>
+        <v>4199</v>
       </c>
       <c r="N81" t="n">
-        <v>0</v>
+        <v>0.003857</v>
       </c>
       <c r="O81" t="n">
-        <v>0</v>
+        <v>0.016797</v>
       </c>
       <c r="P81" t="n">
-        <v>0</v>
+        <v>0.020654</v>
       </c>
     </row>
     <row r="82">
@@ -8245,12 +8506,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>Reaco - 2022 Auto - LR_20-22.pdf</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8260,45 +8521,45 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>1-23</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="G82" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>14.83</v>
+        <v>14.59</v>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
+        <v>5851</v>
       </c>
       <c r="K82" t="n">
-        <v>0</v>
+        <v>1327</v>
       </c>
       <c r="L82" t="n">
-        <v>0</v>
+        <v>5851</v>
       </c>
       <c r="M82" t="n">
-        <v>0</v>
+        <v>1327</v>
       </c>
       <c r="N82" t="n">
-        <v>0</v>
+        <v>0.00117</v>
       </c>
       <c r="O82" t="n">
-        <v>0</v>
+        <v>0.001062</v>
       </c>
       <c r="P82" t="n">
-        <v>0</v>
+        <v>0.002232</v>
       </c>
     </row>
     <row r="83">
@@ -8309,12 +8570,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Reaco - 2022 WC - LR.pdf</t>
+          <t>Reaco - 2022 Auto - LR_20-22.pdf</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8329,40 +8590,40 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>1-23</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I83" t="n">
-        <v>44.87</v>
+        <v>34.51</v>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
+        <v>6164</v>
       </c>
       <c r="K83" t="n">
-        <v>0</v>
+        <v>4601</v>
       </c>
       <c r="L83" t="n">
-        <v>0</v>
+        <v>6164</v>
       </c>
       <c r="M83" t="n">
-        <v>0</v>
+        <v>4601</v>
       </c>
       <c r="N83" t="n">
-        <v>0</v>
+        <v>0.001233</v>
       </c>
       <c r="O83" t="n">
-        <v>0</v>
+        <v>0.003681</v>
       </c>
       <c r="P83" t="n">
-        <v>0</v>
+        <v>0.004914</v>
       </c>
     </row>
     <row r="84">
@@ -8378,7 +8639,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>qa</t>
+          <t>layout</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8388,45 +8649,45 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>chunk 1/1</t>
+          <t>layout discovery</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>1-23</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="G84" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>49.66</v>
+        <v>23.95</v>
       </c>
       <c r="J84" t="n">
-        <v>0</v>
+        <v>19042</v>
       </c>
       <c r="K84" t="n">
-        <v>0</v>
+        <v>1933</v>
       </c>
       <c r="L84" t="n">
-        <v>0</v>
+        <v>3808</v>
       </c>
       <c r="M84" t="n">
-        <v>0</v>
+        <v>387</v>
       </c>
       <c r="N84" t="n">
-        <v>0</v>
+        <v>0.003808</v>
       </c>
       <c r="O84" t="n">
-        <v>0</v>
+        <v>0.001546</v>
       </c>
       <c r="P84" t="n">
-        <v>0</v>
+        <v>0.005355</v>
       </c>
     </row>
     <row r="85">
@@ -8437,12 +8698,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>WC Loss Runs.pdf</t>
+          <t>Reaco - 2022 WC - LR.pdf</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>extract</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8452,16 +8713,16 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>layout discovery</t>
+          <t>chunk 1/1</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-23</t>
         </is>
       </c>
       <c r="G85" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
@@ -8469,28 +8730,28 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>20.23</v>
+        <v>203.15</v>
       </c>
       <c r="J85" t="n">
-        <v>18123</v>
+        <v>70534</v>
       </c>
       <c r="K85" t="n">
-        <v>1945</v>
+        <v>31184</v>
       </c>
       <c r="L85" t="n">
-        <v>3625</v>
+        <v>3067</v>
       </c>
       <c r="M85" t="n">
-        <v>389</v>
+        <v>1356</v>
       </c>
       <c r="N85" t="n">
-        <v>0.003625</v>
+        <v>0.014107</v>
       </c>
       <c r="O85" t="n">
-        <v>0.001556</v>
+        <v>0.024947</v>
       </c>
       <c r="P85" t="n">
-        <v>0.005181</v>
+        <v>0.039054</v>
       </c>
     </row>
     <row r="86">
@@ -8501,59 +8762,443 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
+          <t>Reaco - 2022 WC - LR.pdf</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>23</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>104.97</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Reaco - 2022 WC - LR.pdf</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>23</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>136.66</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Reaco - 2022 WC - LR.pdf</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>23</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0</v>
+      </c>
+      <c r="P88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Reaco - 2022 WC - LR.pdf</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>23</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>44.87</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Reaco - 2022 WC - LR.pdf</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>qa</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>chunk 1/1</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>23</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>49.66</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0</v>
+      </c>
+      <c r="P90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>WC Loss Runs.pdf</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>layout</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>openai/gpt-5.6-luna</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>layout discovery</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>5</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>20.23</v>
+      </c>
+      <c r="J91" t="n">
+        <v>18123</v>
+      </c>
+      <c r="K91" t="n">
+        <v>1945</v>
+      </c>
+      <c r="L91" t="n">
+        <v>3625</v>
+      </c>
+      <c r="M91" t="n">
+        <v>389</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0.003625</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.001556</v>
+      </c>
+      <c r="P91" t="n">
+        <v>0.005181</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>new24</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>WC Loss Runs.pdf</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
         <is>
           <t>extract</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>openai/gpt-5.6-luna</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>chunk 1/1</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>1-6</t>
         </is>
       </c>
-      <c r="G86" t="n">
+      <c r="G92" t="n">
         <v>6</v>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H92" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="I86" t="n">
+      <c r="I92" t="n">
         <v>132.49</v>
       </c>
-      <c r="J86" t="n">
+      <c r="J92" t="n">
         <v>21214</v>
       </c>
-      <c r="K86" t="n">
+      <c r="K92" t="n">
         <v>19486</v>
       </c>
-      <c r="L86" t="n">
+      <c r="L92" t="n">
         <v>3536</v>
       </c>
-      <c r="M86" t="n">
+      <c r="M92" t="n">
         <v>3248</v>
       </c>
-      <c r="N86" t="n">
+      <c r="N92" t="n">
         <v>0.004243</v>
       </c>
-      <c r="O86" t="n">
+      <c r="O92" t="n">
         <v>0.015589</v>
       </c>
-      <c r="P86" t="n">
+      <c r="P92" t="n">
         <v>0.019832</v>
       </c>
     </row>

</xml_diff>